<commit_message>
chore: update Instagram report 2026-08-29 06:52
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -74,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -86,9 +86,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -484,7 +481,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-08-27 13:47:19</t>
+          <t>取得日時：2026-08-29 06:52:55</t>
         </is>
       </c>
     </row>
@@ -496,7 +493,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-08-26</t>
+          <t>比較基準：2026-08-28 保存記録なし</t>
         </is>
       </c>
     </row>
@@ -674,27 +671,27 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>288</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>+4件</t>
+          <t>294</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>530</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+          <t>531</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26T23:00:02+0000</t>
+          <t>2026-08-28T12:10:08+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -731,7 +728,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -741,7 +738,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -783,7 +780,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -793,7 +790,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -803,12 +800,12 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -934,12 +931,12 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>-1件</t>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -947,19 +944,19 @@
           <t>103</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>+0人</t>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24T10:25:05+0000</t>
+          <t>2026-08-28T10:30:06+0000</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1095,7 +1092,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1105,7 +1102,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1197,9 +1194,9 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>+0件</t>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1207,9 +1204,9 @@
           <t>551</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>-1人</t>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1216,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1530</t>
+          <t>1532</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1249,9 +1246,9 @@
           <t>52</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>+0件</t>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -1259,9 +1256,9 @@
           <t>339</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1268,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,12 +1295,12 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>+2件</t>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1311,14 +1308,14 @@
           <t>225</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>+3人</t>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26T10:20:04+0000</t>
+          <t>2026-08-28T12:11:27+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1350,32 +1347,32 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>78</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26T11:00:07+0000</t>
+          <t>2026-08-27T11:00:07+0000</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1402,37 +1399,37 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>2026-08-23T11:23:21+0000</t>
+          <t>2026-08-27T09:03:57+0000</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1457,9 +1454,9 @@
           <t>8</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>+2件</t>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -1467,9 +1464,9 @@
           <t>313</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -1479,7 +1476,7 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -1509,19 +1506,19 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>74</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1528,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1558,42 +1555,42 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>156</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19T10:46:32+0000</t>
+          <t>2026-08-27T09:37:13+0000</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>凡例：🟢 直近3日未満 / 🟡 3〜6日 / 🔴 7日以上 / ⚪ API取得不可</t>
         </is>

</xml_diff>

<commit_message>
chore: update Instagram report 2026-08-30 05:53
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -74,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -86,6 +86,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -481,19 +484,19 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-08-29 06:52:55</t>
+          <t>取得日時：2026-08-30 05:53:30</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>取得成功：13/20</t>
+          <t>取得成功：12/20</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-08-28 保存記録なし</t>
+          <t>比較基準：2026-08-29</t>
         </is>
       </c>
     </row>
@@ -671,12 +674,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>294</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
+          <t>297</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>+3件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -684,14 +687,14 @@
           <t>531</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28T12:10:08+0000</t>
+          <t>2026-08-29T12:10:08+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -728,7 +731,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>算出不可</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -738,7 +741,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>算出不可</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -780,7 +783,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>算出不可</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -790,7 +793,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>算出不可</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -800,7 +803,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -936,7 +939,7 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>算出不可</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -946,7 +949,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>算出不可</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -956,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1092,7 +1095,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>算出不可</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1102,7 +1105,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>算出不可</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1194,19 +1197,19 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>551</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
+          <t>550</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1216,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1532</t>
+          <t>1533</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1243,12 +1246,12 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>52</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -1256,24 +1259,24 @@
           <t>339</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-23T11:06:19+0000</t>
+          <t>2026-08-29T10:59:50+0000</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1295,27 +1298,27 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>52</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>+3件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>225</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
+          <t>224</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28T12:11:27+0000</t>
+          <t>2026-08-29T12:37:27+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1352,7 +1355,7 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>算出不可</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1362,7 +1365,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>算出不可</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1372,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1399,32 +1402,32 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>+4人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27T09:03:57+0000</t>
+          <t>2026-08-29T14:28:24+0000</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1451,7 +1454,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -1461,7 +1464,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>313</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1471,17 +1474,17 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26T11:40:44+0000</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -1506,19 +1509,19 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1528,12 +1531,12 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1555,32 +1558,32 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>156</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
+          <t>159</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>+3人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27T09:37:13+0000</t>
+          <t>2026-08-29T11:07:12+0000</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -1590,7 +1593,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>凡例：🟢 直近3日未満 / 🟡 3〜6日 / 🔴 7日以上 / ⚪ API取得不可</t>
         </is>

</xml_diff>

<commit_message>
chore: update Instagram report 2026-08-31 00:58
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-08-30 06:43:08</t>
+          <t>取得日時：2026-08-31 00:58:56</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-08-29</t>
+          <t>比較基準：2026-08-30</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>297</t>
+          <t>300</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,17 +684,17 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>531</t>
+          <t>532</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29T12:10:08+0000</t>
+          <t>2026-08-30T12:10:08+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -729,19 +729,19 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -778,37 +778,37 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25T14:46:07+0000</t>
+          <t>2026-08-30T14:40:46+0000</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1093,19 +1093,19 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1204,12 +1204,12 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>551</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>-1人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1249,9 +1249,9 @@
           <t>53</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -1259,7 +1259,7 @@
           <t>339</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>58</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -1308,17 +1308,17 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>224</t>
+          <t>226</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>-1人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29T12:37:27+0000</t>
+          <t>2026-08-30T03:49:20+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1353,19 +1353,19 @@
           <t>29</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>81</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,12 +1375,12 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1402,27 +1402,27 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+2件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>43</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>+4人</t>
+          <t>+5人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29T14:28:24+0000</t>
+          <t>2026-08-30T13:07:34+0000</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -1509,7 +1509,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1519,9 +1519,9 @@
           <t>76</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1563,17 +1563,17 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>161</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>+3人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-01 05:53
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-08-31 06:43:03</t>
+          <t>取得日時：2026-09-01 05:53:42</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-08-30</t>
+          <t>比較基準：2026-08-31</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>303</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -689,12 +689,12 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-30T12:10:08+0000</t>
+          <t>2026-08-31T12:10:19+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -778,37 +778,37 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>算出不可</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-30T14:40:46+0000</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>⚪</t>
         </is>
       </c>
     </row>
@@ -959,12 +959,12 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1093,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1103,9 +1103,9 @@
           <t>2</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>31</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>⚪</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>552</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1534</t>
+          <t>1535</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1246,32 +1246,32 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>53</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>339</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>340</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29T10:59:50+0000</t>
+          <t>2026-08-31T15:47:31+0000</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1303,17 +1303,17 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+3件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>227</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>83</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1405,9 +1405,9 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>+2件</t>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1415,9 +1415,9 @@
           <t>43</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>+5人</t>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,19 +1509,19 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>76</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1568,12 +1568,12 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>164</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>+3人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-02 05:54
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-01 06:43:23</t>
+          <t>取得日時：2026-09-02 05:54:34</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-08-31</t>
+          <t>比較基準：2026-09-01</t>
         </is>
       </c>
     </row>
@@ -674,27 +674,27 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>304</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+3件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>533</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31T12:10:19+0000</t>
+          <t>2026-09-01T12:10:37+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -729,7 +729,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -739,9 +739,9 @@
           <t>8</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,37 +1090,37 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>+5人</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-01T10:05:03+0000</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1142,37 +1142,37 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>+6人</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-31T21:48:11+0000</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>算出不可</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>552</t>
+          <t>553</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1535</t>
+          <t>1536</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>55</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -1261,12 +1261,12 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31T15:47:31+0000</t>
+          <t>2026-09-01T09:59:50+0000</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -1308,12 +1308,12 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>227</t>
+          <t>229</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1353,7 +1353,7 @@
           <t>29</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1363,9 +1363,9 @@
           <t>83</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1405,19 +1405,19 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>43</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,7 +1509,7 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1519,9 +1519,9 @@
           <t>78</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1561,7 +1561,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1571,9 +1571,9 @@
           <t>164</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,12 +1583,12 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-03 05:55
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-02 06:45:26</t>
+          <t>取得日時：2026-09-03 05:55:37</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-01</t>
+          <t>比較基準：2026-09-02</t>
         </is>
       </c>
     </row>
@@ -679,12 +679,12 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>533</t>
+          <t>534</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -934,37 +934,37 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>103</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>104</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28T10:30:06+0000</t>
+          <t>2026-09-02T10:40:02+0000</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1100,17 +1100,17 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+5人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01T10:05:03+0000</t>
+          <t>2026-09-02T10:08:35+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1152,17 +1152,17 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+6人</t>
+          <t>+3人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31T21:48:11+0000</t>
+          <t>2026-09-02T10:10:47+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1197,7 +1197,7 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1207,9 +1207,9 @@
           <t>553</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1536</t>
+          <t>1537</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1249,9 +1249,9 @@
           <t>55</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -1259,7 +1259,7 @@
           <t>340</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,12 +1298,12 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>61</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+3件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1313,17 +1313,17 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-08-30T03:49:20+0000</t>
+          <t>2026-09-02T09:39:10+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1353,19 +1353,19 @@
           <t>29</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>83</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1402,12 +1402,12 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1417,17 +1417,17 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>2026-08-30T13:07:34+0000</t>
+          <t>2026-09-01T21:56:54+0000</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,19 +1509,19 @@
           <t>6</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>78</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,12 +1531,12 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1561,19 +1561,19 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>164</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>165</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-04 05:54
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-03 06:46:01</t>
+          <t>取得日時：2026-09-04 05:54:09</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-02</t>
+          <t>比較基準：2026-09-03</t>
         </is>
       </c>
     </row>
@@ -674,17 +674,17 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>304</t>
+          <t>305</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>534</t>
+          <t>535</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -694,12 +694,12 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01T12:10:37+0000</t>
+          <t>2026-09-02T23:06:08+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -949,12 +949,12 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02T10:40:02+0000</t>
+          <t>2026-09-03T10:40:02+0000</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02T10:08:35+0000</t>
+          <t>2026-09-03T10:50:07+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>44</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02T10:10:47+0000</t>
+          <t>2026-09-03T10:39:54+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1537</t>
+          <t>1538</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,12 +1298,12 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>62</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+3件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02T09:39:10+0000</t>
+          <t>2026-09-03T00:03:23+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1365,22 +1365,22 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27T11:00:07+0000</t>
+          <t>2026-09-03T11:08:22+0000</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1405,9 +1405,9 @@
           <t>7</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1415,7 +1415,7 @@
           <t>44</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1506,17 +1506,17 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>80</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -1526,17 +1526,17 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26T13:20:04+0000</t>
+          <t>2026-09-03T07:07:36+0000</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🔴</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>166</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-05 05:53
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-04 06:44:13</t>
+          <t>取得日時：2026-09-05 05:53:34</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-03</t>
+          <t>比較基準：2026-09-04</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>305</t>
+          <t>311</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+6件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -689,12 +689,12 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02T23:06:08+0000</t>
+          <t>2026-09-04T12:10:06+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03T10:40:02+0000</t>
+          <t>2026-09-04T10:40:01+0000</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1100,17 +1100,17 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03T10:50:07+0000</t>
+          <t>2026-09-04T10:01:14+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+3人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03T10:39:54+0000</t>
+          <t>2026-09-04T09:42:25+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1538</t>
+          <t>1539</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1249,19 +1249,19 @@
           <t>55</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>340</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>341</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1298,12 +1298,12 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>65</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+3件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03T00:03:23+0000</t>
+          <t>2026-09-04T07:35:05+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1355,17 +1355,17 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>83</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1402,12 +1402,12 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1415,19 +1415,19 @@
           <t>44</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01T21:56:54+0000</t>
+          <t>2026-09-04T10:39:23+0000</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1511,12 +1511,12 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>81</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>166</t>
+          <t>167</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-06 05:54
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-05 06:44:43</t>
+          <t>取得日時：2026-09-06 05:54:12</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-04</t>
+          <t>比較基準：2026-09-05</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>311</t>
+          <t>316</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+6件</t>
+          <t>+5件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04T12:10:06+0000</t>
+          <t>2026-09-05T12:10:16+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -729,19 +729,19 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04T10:40:01+0000</t>
+          <t>2026-09-05T10:21:10+0000</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04T10:01:14+0000</t>
+          <t>2026-09-05T12:00:04+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04T09:42:25+0000</t>
+          <t>2026-09-05T12:01:29+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1539</t>
+          <t>1540</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1246,17 +1246,17 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>57</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+2件</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>341</t>
+          <t>342</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -1266,17 +1266,17 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01T09:59:50+0000</t>
+          <t>2026-09-05T16:07:28+0000</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1298,27 +1298,27 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>69</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+3件</t>
+          <t>+4件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>230</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04T07:35:05+0000</t>
+          <t>2026-09-05T09:53:43+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1360,12 +1360,12 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>84</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>-1人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1407,17 +1407,17 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1506,17 +1506,17 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+2件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>82</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -1526,12 +1526,12 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03T07:07:36+0000</t>
+          <t>2026-09-05T12:31:05+0000</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1558,22 +1558,22 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>167</t>
+          <t>171</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+4人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,12 +1583,12 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-07 05:53
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-06 06:43:11</t>
+          <t>取得日時：2026-09-07 05:53:56</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-05</t>
+          <t>比較基準：2026-09-06</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>316</t>
+          <t>321</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,17 +684,17 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>535</t>
+          <t>536</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-05T12:10:16+0000</t>
+          <t>2026-09-06T12:10:08+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -729,7 +729,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -739,9 +739,9 @@
           <t>10</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -939,17 +939,17 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1095,12 +1095,12 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1145,9 +1145,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1155,7 +1155,7 @@
           <t>44</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1540</t>
+          <t>1541</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1251,17 +1251,17 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>+2件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>342</t>
+          <t>341</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,17 +1298,17 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>72</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+4件</t>
+          <t>+3件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>231</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-05T09:53:43+0000</t>
+          <t>2026-09-06T06:30:05+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1360,12 +1360,12 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>82</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>-2人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,12 +1375,12 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1402,12 +1402,12 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1417,17 +1417,17 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04T10:39:23+0000</t>
+          <t>2026-09-06T14:22:00+0000</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,9 +1509,9 @@
           <t>9</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>+2件</t>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1519,9 +1519,9 @@
           <t>82</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1561,9 +1561,9 @@
           <t>11</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1571,9 +1571,9 @@
           <t>171</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>+4人</t>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-08 05:54
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-07 06:43:41</t>
+          <t>取得日時：2026-09-08 05:54:59</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-06</t>
+          <t>比較基準：2026-09-07</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>326</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,17 +684,17 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>536</t>
+          <t>538</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-06T12:10:08+0000</t>
+          <t>2026-09-07T12:10:07+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -729,19 +729,19 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>+7人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -937,7 +937,7 @@
           <t>32</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -947,9 +947,9 @@
           <t>105</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1145,19 +1145,19 @@
           <t>5</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1541</t>
+          <t>1542</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1256,12 +1256,12 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>341</t>
+          <t>342</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>-1人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1303,12 +1303,12 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+3件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>231</t>
+          <t>232</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1350,37 +1350,37 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>83</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>-2人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03T11:08:22+0000</t>
+          <t>2026-09-07T03:25:00+0000</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -1412,17 +1412,17 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>47</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>2026-09-06T14:22:00+0000</t>
+          <t>2026-09-07T12:41:19+0000</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -1509,19 +1509,19 @@
           <t>9</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>82</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1561,19 +1561,19 @@
           <t>11</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>171</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>172</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-09 05:56
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-08 06:45:50</t>
+          <t>取得日時：2026-09-09 05:56:26</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-07</t>
+          <t>比較基準：2026-09-08</t>
         </is>
       </c>
     </row>
@@ -674,12 +674,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>326</t>
+          <t>329</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>+5件</t>
+          <t>+3件</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -689,12 +689,12 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07T12:10:07+0000</t>
+          <t>2026-09-08T12:10:07+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -736,12 +736,12 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>+7人</t>
+          <t>+3人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -959,12 +959,12 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1090,12 +1090,12 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1105,17 +1105,17 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-05T12:00:04+0000</t>
+          <t>2026-09-08T10:26:58+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1142,17 +1142,17 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>48</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -1162,12 +1162,12 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-05T12:01:29+0000</t>
+          <t>2026-09-08T10:26:27+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1197,19 +1197,19 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>553</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1542</t>
+          <t>1543</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1249,7 +1249,7 @@
           <t>57</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1259,9 +1259,9 @@
           <t>342</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
           <t>72</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1311,9 +1311,9 @@
           <t>232</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>+1件</t>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>84</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1405,9 +1405,9 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1415,9 +1415,9 @@
           <t>47</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,7 +1509,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1519,9 +1519,9 @@
           <t>84</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>+2人</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,12 +1531,12 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
           <t>11</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1571,9 +1571,9 @@
           <t>172</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-10 05:54
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-09 06:45:43</t>
+          <t>取得日時：2026-09-10 05:54:33</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-08</t>
+          <t>比較基準：2026-09-09</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>332</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,17 +684,17 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>538</t>
+          <t>537</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08T12:10:07+0000</t>
+          <t>2026-09-09T12:10:05+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -729,7 +729,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -739,9 +739,9 @@
           <t>20</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>+3人</t>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1100,17 +1100,17 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08T10:26:58+0000</t>
+          <t>2026-09-09T10:28:07+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08T10:26:27+0000</t>
+          <t>2026-09-09T10:29:17+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1197,7 +1197,7 @@
           <t>42</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1207,9 +1207,9 @@
           <t>554</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1543</t>
+          <t>1544</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1249,19 +1249,19 @@
           <t>57</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>342</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>343</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,12 +1298,12 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>72</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>+4件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1311,19 +1311,19 @@
           <t>232</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-06T06:30:05+0000</t>
+          <t>2026-09-09T08:47:08+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -1353,7 +1353,7 @@
           <t>31</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1363,9 +1363,9 @@
           <t>84</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,19 +1509,19 @@
           <t>9</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-11 05:55
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-10 06:45:49</t>
+          <t>取得日時：2026-09-11 05:55:17</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-09</t>
+          <t>比較基準：2026-09-10</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>332</t>
+          <t>335</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,17 +684,17 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>537</t>
+          <t>538</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>-1人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09T12:10:05+0000</t>
+          <t>2026-09-10T12:10:07+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -729,19 +729,19 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>+0人</t>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1100,17 +1100,17 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>19</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+3人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09T10:28:07+0000</t>
+          <t>2026-09-10T10:40:11+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1152,17 +1152,17 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>50</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09T10:29:17+0000</t>
+          <t>2026-09-10T10:50:57+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1544</t>
+          <t>1545</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1256,12 +1256,12 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>343</t>
+          <t>345</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+2人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,12 +1298,12 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>79</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+4件</t>
+          <t>+3件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09T08:47:08+0000</t>
+          <t>2026-09-10T06:55:08+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1350,12 +1350,12 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1363,19 +1363,19 @@
           <t>84</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07T03:25:00+0000</t>
+          <t>2026-09-09T22:57:15+0000</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,12 +1427,12 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>🟢</t>
+          <t>🟡</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>86</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-12 05:55
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-11 06:45:30</t>
+          <t>取得日時：2026-09-12 05:55:40</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-10</t>
+          <t>比較基準：2026-09-11</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>335</t>
+          <t>338</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,17 +684,17 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>538</t>
+          <t>537</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10T12:10:07+0000</t>
+          <t>2026-09-11T12:10:06+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -736,12 +736,12 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1100,17 +1100,17 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+3人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10T10:40:11+0000</t>
+          <t>2026-09-11T10:18:02+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10T10:50:57+0000</t>
+          <t>2026-09-11T10:39:26+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1545</t>
+          <t>1546</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1256,12 +1256,12 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>345</t>
+          <t>346</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>+2人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1298,27 +1298,27 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>81</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>+3件</t>
+          <t>+2件</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>231</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>+0人</t>
+          <t>-1人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10T06:55:08+0000</t>
+          <t>2026-09-11T07:41:24+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1353,9 +1353,9 @@
           <t>32</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>+1件</t>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>+0件</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1363,7 +1363,7 @@
           <t>84</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1516,12 +1516,12 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>89</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+3人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: update Instagram report 2026-09-13 05:56
</commit_message>
<xml_diff>
--- a/instagram-daily-checker/reports/latest.xlsx
+++ b/instagram-daily-checker/reports/latest.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>取得日時：2026-09-12 06:44:15</t>
+          <t>取得日時：2026-09-13 05:56:16</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>比較基準：2026-09-11</t>
+          <t>比較基準：2026-09-12</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>338</t>
+          <t>341</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>537</t>
+          <t>536</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11T12:10:06+0000</t>
+          <t>2026-09-12T12:10:07+0000</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -729,7 +729,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -739,9 +739,9 @@
           <t>23</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>+1人</t>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -934,12 +934,12 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>+0件</t>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -947,24 +947,24 @@
           <t>105</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>+0人</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>2026-09-05T10:21:10+0000</t>
+          <t>2026-09-12T10:15:02+0000</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1105,12 +1105,12 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11T10:18:02+0000</t>
+          <t>2026-09-12T13:30:22+0000</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11T10:39:26+0000</t>
+          <t>2026-09-12T15:25:04+0000</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1546</t>
+          <t>1547</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1246,12 +1246,12 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>58</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>+0件</t>
+          <t>+1件</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -1261,22 +1261,22 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>+1人</t>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-05T16:07:28+0000</t>
+          <t>2026-09-12T12:52:38+0000</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🟢</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>83</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -1308,17 +1308,17 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>231</t>
+          <t>232</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>-1人</t>
+          <t>+1人</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11T07:41:24+0000</t>
+          <t>2026-09-12T05:40:05+0000</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1509,7 +1509,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>+0件</t>
         </is>
@@ -1519,9 +1519,9 @@
           <t>89</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>+3人</t>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+0人</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1531,12 +1531,12 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>🟡</t>
+          <t>🔴</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">

</xml_diff>